<commit_message>
Automation landing: rebuild in the homepage's calm single-screen language (big stat, one claim, TEXT US); keep Codex version as automation-codex.html
</commit_message>
<xml_diff>
--- a/Agripals Caller - Target Accounts.xlsx
+++ b/Agripals Caller - Target Accounts.xlsx
@@ -68,7 +68,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +83,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -156,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -175,6 +180,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1746,2407 +1754,3020 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:H103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Companies extracted from uploaded client-wall logo images (18 Jul 2026)</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Agripals Caller — Client Wall Prospects, enriched (Australian ag-adjacent orgs from client-wall logos)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>These appear to be past research clients, not verified Agripals Caller prospects. Category is best-guess from the company name/logo. No contact details researched yet — verify before outreach.</t>
+          <t>Source: uploaded client-wall logo images, likely past clients of an agricultural market-research firm — not existing Agripals customers. Researched 18 Jul 2026. Fit is noted honestly, including "weak/unclear" where applicable.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Segment</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Organisation</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>First Name</t>
+          <t>Status / M&amp;A note</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Surname</t>
+          <t>Why they'd buy (or fit note)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Company</t>
+          <t>Contact route (URL)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Contact Number</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Comments / Notes</t>
+          <t>Confidence</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Achmea</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr"/>
-      <c r="I5" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ag chem / input suppliers</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>University/Research</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
+          <t>BASF (BASF Crop Solutions)</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Agchem input supplier — plausible buyer of grower survey/market-research data.</t>
+        </is>
+      </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>ACFR (Australian Centre for Field Robotics)</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr"/>
-      <c r="I6" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://www.basf.com/au/en/who-we-are/sites-and-contacts</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>agro-ANZ@basf.com</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>1800 558 399</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Machinery</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
+          <t>Bayer Crop Science Australia</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Agchem/seed input supplier — same rationale as BASF.</t>
+        </is>
+      </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>AGCO</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://www.crop.bayer.com.au/contact-us</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>aust.cs@bayer.com</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>1800 636 001</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Industry Body</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr"/>
-      <c r="D8" s="7" t="inlineStr"/>
+          <t>BioAg</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — Riverina, NSW.</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Biological fertiliser company — could use grower feedback/survey data.</t>
+        </is>
+      </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>AMPC (Australian Meat Processor Corporation)</t>
+          <t>https://bioag.com.au/</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr"/>
       <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Partial — only regional sales-manager emails found</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Industry Body</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr"/>
-      <c r="D9" s="7" t="inlineStr"/>
+          <t>CSBP</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — part of Wesfarmers Chemicals, Energy &amp; Fertilisers.</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>WA fertiliser/chemicals business with existing AgTech (DecipherAg) arm — plausible buyer of grower data services.</t>
+        </is>
+      </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Animal Health Australia</t>
+          <t>https://csbp.com.au/support/contact-us/head-office/</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>1800 808 728</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Bank</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr"/>
-      <c r="D10" s="7" t="inlineStr"/>
+          <t>Dow (ag business)</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Ag division merged into Corteva Agriscience (DowDuPont split, Jun 2019).</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Global crop-input company via Corteva — could commission grower feedback/product-adoption surveys.</t>
+        </is>
+      </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>ANZ</t>
+          <t>https://corteva.com/au/contact-us.html</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>1800 700 096</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr"/>
-      <c r="D11" s="7" t="inlineStr"/>
+          <t>DuPont (ag business)</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Ag division merged into Corteva Agriscience; DuPont continues separately in non-ag specialty chemicals.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Same rationale as Dow, via Corteva.</t>
+        </is>
+      </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>AUSTAR</t>
+          <t>https://corteva.com/au/contact-us.html</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr"/>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>1800 700 096</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Industry Body</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr"/>
-      <c r="D12" s="7" t="inlineStr"/>
+          <t>Incitec Pivot Fertilisers</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Parent Incitec Pivot Ltd renamed Dyno Nobel (Mar 2025); fertiliser distribution business sold to Ridley Corporation (completed Sep 2025), still trades as Incitec Pivot Fertilisers.</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Fertiliser distributor — could commission grower survey/usage data.</t>
+        </is>
+      </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Australian Eggs</t>
+          <t>https://incitecpivot.com.au/contact-us/</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr"/>
       <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Govt</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr"/>
-      <c r="D13" s="7" t="inlineStr"/>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>Centrelink</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>Novozymes</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Merged with Chr. Hansen (Jan 2024) to form Novonesis.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Industrial enzymes/biotech — weak/unclear fit, though could commission ag-input adoption research.</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>aucustomerservice@novonesis.com</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>+61 3 9762 9600</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Govt</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr"/>
-      <c r="D14" s="7" t="inlineStr"/>
+          <t>Nufarm</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged (ASX-listed).</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Agrochemical company — plausible buyer of grower product-usage/feedback phone surveys.</t>
+        </is>
+      </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Department of Agriculture, Fisheries and Forestry (Cwlth)</t>
+          <t>https://nufarm.com/contact/</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
-      <c r="I14" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>(61-3) 9282 1000</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Grain</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr"/>
-      <c r="D15" s="7" t="inlineStr"/>
+          <t>Sinochem Australia</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged (Kelpie, Roundup licensing).</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Agrochemical supplier — could commission grower product-performance surveys.</t>
+        </is>
+      </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>AWB</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr"/>
+          <t>https://www.sinochem.com.au/support/contact-us/</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>customerservice@kelpiecp.com</t>
+        </is>
+      </c>
       <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Ag Chem</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr"/>
-      <c r="D16" s="7" t="inlineStr"/>
+          <t>Sumitomo Chemical Australia</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Agrochemical company — grower product-feedback/research surveys plausible.</t>
+        </is>
+      </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>https://www.sumitomo-chem.com.au/contact-us</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr"/>
-      <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
-      <c r="I16" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>+61 2 8752 9000</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Ag Chem</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr"/>
-      <c r="D17" s="7" t="inlineStr"/>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Bayer</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr"/>
-      <c r="G17" s="7" t="inlineStr"/>
-      <c r="H17" s="7" t="inlineStr"/>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr"/>
-      <c r="D18" s="7" t="inlineStr"/>
+          <t>AGCO</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — Massey Ferguson, Fendt, Valtra.</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Farm equipment manufacturer — dealer/customer satisfaction surveys plausible.</t>
+        </is>
+      </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>BHP Billiton</t>
+          <t>https://www.agcocorp.com/us/en/home/contact.html</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr"/>
-      <c r="G18" s="7" t="inlineStr"/>
-      <c r="H18" s="7" t="inlineStr"/>
-      <c r="I18" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>+61 3 9313 0313</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Ag Chem</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr"/>
-      <c r="D19" s="7" t="inlineStr"/>
+          <t>Case IH</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — brand of CNH Industrial.</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Farm equipment brand — dealer/customer survey use case.</t>
+        </is>
+      </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>BioAg</t>
+          <t>https://www.caseih.com/en-au/australia/connect-with-us/contact-us</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr"/>
       <c r="G19" s="7" t="inlineStr"/>
-      <c r="H19" s="7" t="inlineStr"/>
-      <c r="I19" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr"/>
-      <c r="D20" s="7" t="inlineStr"/>
+          <t>John Deere</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged (Deere &amp; Company).</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Machinery OEM — plausible buyer of structured farmer feedback/market research.</t>
+        </is>
+      </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Caltex Australia</t>
+          <t>https://www.deere.com.au/en/our-company/contact-us/</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr"/>
-      <c r="G20" s="7" t="inlineStr"/>
-      <c r="H20" s="7" t="inlineStr"/>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>1800 800 981</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Grain</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr"/>
-      <c r="D21" s="7" t="inlineStr"/>
+          <t>Philmac</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — subsidiary of global group Aliaxis.</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Irrigation/poly-pipe fittings manufacturer — could commission on-farm irrigation-practice surveys.</t>
+        </is>
+      </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Cargill</t>
+          <t>https://philmac.com.au/company/</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr"/>
       <c r="G21" s="7" t="inlineStr"/>
-      <c r="H21" s="7" t="inlineStr"/>
-      <c r="I21" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Machinery</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr"/>
-      <c r="D22" s="7" t="inlineStr"/>
+          <t>Silvan</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — farm/horticultural sprayer manufacturer since 1962.</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Equipment manufacturer — dealer/customer satisfaction surveys conceivable, not core to business.</t>
+        </is>
+      </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Case IH</t>
+          <t>https://www.silvan.com.au/contact/</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr"/>
       <c r="G22" s="7" t="inlineStr"/>
-      <c r="H22" s="7" t="inlineStr"/>
-      <c r="I22" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Research/Market Research</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr"/>
-      <c r="D23" s="7" t="inlineStr"/>
+          <t>Tapex (Tapex Group)</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Industrial twine/protective packaging incl. ag/silage products — weak fit as a data-services buyer.</t>
+        </is>
+      </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
+          <t>https://tapexgroup.com.au/contact-us/</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>enquiries@tapexgroup.com.au</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>+61 2 9502 6000</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Toyota Australia</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Strong rural/farmer customer base (HiLux, LandCruiser) — Toyota for Business could commission rural customer research.</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>https://www.toyota.com.au/support/contact-us</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr"/>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>1800 869 682 / 1800 679 247 (Business)</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Achmea (Achmea Farm Insurance)</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — Dutch-owned specialist farm insurer.</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Insurer needing structured claims/risk data collection from farmers.</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>https://www.achmea.com.au/contact-us/</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>claims@achmea.com.au</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>1800 724 214</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>CGU</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — brand of Insurance Australia Group (IAG); offers Farm Insurance.</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Insurer with dedicated farm/crop/livestock cover — plausible buyer of claims/risk survey data.</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>https://www.cgu.com.au/contact</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr"/>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>1300 943 690</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="7" t="inlineStr">
+        <is>
           <t>CelsiusPro</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr"/>
-      <c r="G23" s="7" t="inlineStr"/>
-      <c r="H23" s="7" t="inlineStr"/>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr"/>
-      <c r="D24" s="7" t="inlineStr"/>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>CGU</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr"/>
-      <c r="G24" s="7" t="inlineStr"/>
-      <c r="H24" s="7" t="inlineStr"/>
-      <c r="I24" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Grain</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr"/>
-      <c r="D25" s="7" t="inlineStr"/>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>Clear Grain Exchange</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr"/>
-      <c r="G25" s="7" t="inlineStr"/>
-      <c r="H25" s="7" t="inlineStr"/>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Bank</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr"/>
-      <c r="D26" s="7" t="inlineStr"/>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>Commonwealth Bank</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr"/>
-      <c r="G26" s="7" t="inlineStr"/>
-      <c r="H26" s="7" t="inlineStr"/>
-      <c r="I26" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Supplies</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr"/>
-      <c r="D27" s="7" t="inlineStr"/>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>CopRice</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr"/>
-      <c r="G27" s="7" t="inlineStr"/>
-      <c r="H27" s="7" t="inlineStr"/>
-      <c r="I27" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>University/Research</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr"/>
-      <c r="D28" s="7" t="inlineStr"/>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — Swiss-headquartered parametric weather-risk insurer, AU office.</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Parametric ag-weather insurer — close conceptual overlap with structured data collection.</t>
+        </is>
+      </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>CQUniversity Australia</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr"/>
-      <c r="G28" s="7" t="inlineStr"/>
-      <c r="H28" s="7" t="inlineStr"/>
-      <c r="I28" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://www.celsiuspro.com.au/</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>info@celsiuspro.com.au</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>+61 2 9994 8009</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Industry Body</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr"/>
-      <c r="D29" s="7" t="inlineStr"/>
+          <t>Ruralco Insurance</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Ruralco Holdings acquired by Nutrien (2019), rebranded Nutrien Ag Solutions; insurance broking now "Nutrien Ag Solutions Insurance".</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Large rural insurance broker network with farmer customer base — could commission structured producer research.</t>
+        </is>
+      </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
+          <t>https://www.nutrienagsolutions.com.au/insurance</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr"/>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>1800 888 642</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>RGA (RGA Reinsurance Australia)</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged — APRA-regulated life/health reinsurer.</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Life &amp; health reinsurance — weak fit, only tangential link via farmer life/injury insurance underwriting.</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>https://www.rgare.com/global-presence/asia-pacific/australia-and-new-zealand</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr"/>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>(02) 8264 5800</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>WorkCover SA</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Renamed — WorkCover Corporation of SA replaced by ReturnToWorkSA.</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Covers agricultural workers under SA's workers' comp scheme — could commission farm workplace-safety research.</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>https://www.rtwsa.com/</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>info@rtwsa.com</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>13 18 55</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Animal health</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n"/>
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="6" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Novartis Animal Health</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Sold to Eli Lilly's animal-health arm, Elanco, completed 1 Jan 2015 ($5.28B).</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Successor Elanco is a global animal-health company — plausible buyer of vet/producer phone-survey data.</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>https://www.elanco.com/en-au/contact</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>anz-elanco-customer-service@elancoah.com</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>1800 226 324</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Pfizer Animal Health</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Spun off and fully separated 24 Jun 2013 as Zoetis. NOTE: same successor as the Zoetis entry below — avoid duplicate outreach.</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Successor Zoetis is a global animal-health/diagnostics company.</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>https://www.zoetis.com.au/contact-us</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>customerservice.au@zoetis.com</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>1800 963 847</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Virbac</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — livestock and companion animal health, Milperra NSW.</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Livestock producer/vet feedback and product-performance research is a natural use case.</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>https://au.virbac.com/contact</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>info@virbac.com.au</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>(02) 9772 9772</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Zoetis</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — global animal health company (AU office Banyo QLD).</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Livestock health/product-performance data collection is core to their business — plausible buyer.</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>https://www2.zoetis.com.au/contact-us</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>customerservice.au@zoetis.com</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>1800 022 442</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Industry bodies / RDCs</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="6" t="n"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>AMPC (Australian Meat Processor Corporation)</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>RDC-style body that commissions industry surveys/data collection from processor members.</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>https://ampc.com.au/contact-us/</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>admin@ampc.com.au</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>02 8908 5500</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Animal Health Australia</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Biosecurity/disease surveillance body — plausible interest in structured phone data collection from producers.</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>https://animalhealthaustralia.com.au/contact-us/</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr"/>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>1800 675 888</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Australian Eggs</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Rebranded from Australian Egg Corporation Limited (2017), same legal entity.</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>RDC-style marketing/research body — plausible buyer of producer survey services.</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>https://www.australianeggs.org.au/contact-us</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>contact@australianeggs.org.au</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>+61 2 9409 6999</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="7" t="inlineStr">
+        <is>
           <t>CropLife International</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr"/>
-      <c r="G29" s="7" t="inlineStr"/>
-      <c r="H29" s="7" t="inlineStr"/>
-      <c r="I29" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>AgTech</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr"/>
-      <c r="D30" s="7" t="inlineStr"/>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>CropLogic</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="inlineStr"/>
-      <c r="G30" s="7" t="inlineStr"/>
-      <c r="H30" s="7" t="inlineStr"/>
-      <c r="I30" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Ag Chem</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr"/>
-      <c r="D31" s="7" t="inlineStr"/>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>CSBP</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr"/>
-      <c r="G31" s="7" t="inlineStr"/>
-      <c r="H31" s="7" t="inlineStr"/>
-      <c r="I31" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>University/Research</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr"/>
-      <c r="D32" s="7" t="inlineStr"/>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>CSIRO</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr"/>
-      <c r="G32" s="7" t="inlineStr"/>
-      <c r="H32" s="7" t="inlineStr"/>
-      <c r="I32" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>Industry Body</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr"/>
-      <c r="D33" s="7" t="inlineStr"/>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — Brussels-based global body (note: distinct from local affiliate CropLife Australia — confirm which the logo referred to).</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Industry association — could commission member/stakeholder surveys, though global not AU-specific.</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>https://croplife.org/contact/</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>croplife@croplife.org</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>+32 2 542 04 19</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>Dairy Australia</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr"/>
-      <c r="G33" s="7" t="inlineStr"/>
-      <c r="H33" s="7" t="inlineStr"/>
-      <c r="I33" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>Ag Chem</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr"/>
-      <c r="D34" s="7" t="inlineStr"/>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>Dow</t>
-        </is>
-      </c>
-      <c r="F34" s="7" t="inlineStr"/>
-      <c r="G34" s="7" t="inlineStr"/>
-      <c r="H34" s="7" t="inlineStr"/>
-      <c r="I34" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Ag Chem</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr"/>
-      <c r="D35" s="7" t="inlineStr"/>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>DuPont</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr"/>
-      <c r="G35" s="7" t="inlineStr"/>
-      <c r="H35" s="7" t="inlineStr"/>
-      <c r="I35" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>Agribus</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="inlineStr"/>
-      <c r="D36" s="7" t="inlineStr"/>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>Elders</t>
-        </is>
-      </c>
-      <c r="F36" s="7" t="inlineStr"/>
-      <c r="G36" s="7" t="inlineStr"/>
-      <c r="H36" s="7" t="inlineStr"/>
-      <c r="I36" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>AgTech</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr"/>
-      <c r="D37" s="7" t="inlineStr"/>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>FarmBot Monitoring Solutions</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="inlineStr"/>
-      <c r="G37" s="7" t="inlineStr"/>
-      <c r="H37" s="7" t="inlineStr"/>
-      <c r="I37" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>Research/Market Research</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr"/>
-      <c r="D38" s="7" t="inlineStr"/>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>Food Industry People Group</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="inlineStr"/>
-      <c r="G38" s="7" t="inlineStr"/>
-      <c r="H38" s="7" t="inlineStr"/>
-      <c r="I38" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Grain</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr"/>
-      <c r="D39" s="7" t="inlineStr"/>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>GrainCorp</t>
-        </is>
-      </c>
-      <c r="F39" s="7" t="inlineStr"/>
-      <c r="G39" s="7" t="inlineStr"/>
-      <c r="H39" s="7" t="inlineStr"/>
-      <c r="I39" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t>Govt</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="inlineStr"/>
-      <c r="D40" s="7" t="inlineStr"/>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>GRDC</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr"/>
-      <c r="G40" s="7" t="inlineStr"/>
-      <c r="H40" s="7" t="inlineStr"/>
-      <c r="I40" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr"/>
-      <c r="D41" s="7" t="inlineStr"/>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>Greening Australia</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr"/>
-      <c r="G41" s="7" t="inlineStr"/>
-      <c r="H41" s="7" t="inlineStr"/>
-      <c r="I41" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>Supplies</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="inlineStr"/>
-      <c r="D42" s="7" t="inlineStr"/>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — national dairy industry services body.</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>RDC-style body, analogous to AMPC/Australian Eggs — plausible buyer of farmer survey/data-collection services.</t>
+        </is>
+      </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>Heritage Seeds</t>
+          <t>https://www.dairyaustralia.com.au/contact-us</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr"/>
-      <c r="G42" s="7" t="inlineStr"/>
-      <c r="H42" s="7" t="inlineStr"/>
-      <c r="I42" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>1800 004 377</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Tech</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="inlineStr"/>
-      <c r="D43" s="7" t="inlineStr"/>
+          <t>MLA (Meat &amp; Livestock Australia)</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Regularly commissions producer surveys and market intelligence — very plausible buyer.</t>
+        </is>
+      </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>IBM</t>
-        </is>
-      </c>
-      <c r="F43" s="7" t="inlineStr"/>
-      <c r="G43" s="7" t="inlineStr"/>
-      <c r="H43" s="7" t="inlineStr"/>
-      <c r="I43" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://www.mla.com.au/about-mla/contact/</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>info@mla.com.au</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>1800 023 100</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Ag Chem</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr"/>
-      <c r="D44" s="7" t="inlineStr"/>
+          <t>NSW Farmers</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged (NSW Farmers Association).</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>State farmer advocacy/membership body — plausible buyer/partner for structured farmer-voice data (member surveys, advocacy polling).</t>
+        </is>
+      </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>Incitec Pivot Fertilisers</t>
+          <t>https://www.nswfarmers.org.au</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr"/>
-      <c r="G44" s="7" t="inlineStr"/>
-      <c r="H44" s="7" t="inlineStr"/>
-      <c r="I44" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>02 9478 1000</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>AgTech</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr"/>
-      <c r="D45" s="7" t="inlineStr"/>
+          <t>Plant Health Australia</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — national plant biosecurity coordination body.</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Coordinates biosecurity surveillance/reporting across plant industries — plausible buyer of grower phone-survey data.</t>
+        </is>
+      </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>IPSTAR</t>
-        </is>
-      </c>
-      <c r="F45" s="7" t="inlineStr"/>
-      <c r="G45" s="7" t="inlineStr"/>
-      <c r="H45" s="7" t="inlineStr"/>
-      <c r="I45" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://www.planthealthaustralia.com.au/contact/</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>info@phau.com.au</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>+61 2 6215 7700</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Machinery</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="inlineStr"/>
-      <c r="D46" s="7" t="inlineStr"/>
+          <t>Sheep Producers Australia</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — national peak body for sheepmeat producers.</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Same profile as GRDC/wheat bodies — natural buyer of structured producer phone-survey data.</t>
+        </is>
+      </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>John Deere</t>
-        </is>
-      </c>
-      <c r="F46" s="7" t="inlineStr"/>
-      <c r="G46" s="7" t="inlineStr"/>
-      <c r="H46" s="7" t="inlineStr"/>
-      <c r="I46" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://www.sheepproducers.com.au/contactus</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>ceo@sheepproducers.com.au</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>+61 2 6103 0838</t>
+        </is>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Research/Market Research</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr"/>
-      <c r="D47" s="7" t="inlineStr"/>
+          <t>Victorian Farmers Federation</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — peak body since 1979.</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Direct farmer membership base — natural buyer of producer survey/data-collection services.</t>
+        </is>
+      </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>Kantar</t>
-        </is>
-      </c>
-      <c r="F47" s="7" t="inlineStr"/>
+          <t>https://vff.org.au/contact/</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>media@vff.org.au</t>
+        </is>
+      </c>
       <c r="G47" s="7" t="inlineStr"/>
-      <c r="H47" s="7" t="inlineStr"/>
-      <c r="I47" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="inlineStr">
-        <is>
-          <t>Agribus</t>
-        </is>
-      </c>
-      <c r="C48" s="7" t="inlineStr"/>
-      <c r="D48" s="7" t="inlineStr"/>
-      <c r="E48" s="7" t="inlineStr">
-        <is>
-          <t>Landmark</t>
-        </is>
-      </c>
-      <c r="F48" s="7" t="inlineStr"/>
-      <c r="G48" s="7" t="inlineStr"/>
-      <c r="H48" s="7" t="inlineStr"/>
-      <c r="I48" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Government / statutory</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n"/>
+      <c r="C48" s="5" t="n"/>
+      <c r="D48" s="5" t="n"/>
+      <c r="E48" s="5" t="n"/>
+      <c r="F48" s="5" t="n"/>
+      <c r="G48" s="5" t="n"/>
+      <c r="H48" s="6" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Tech</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="inlineStr"/>
-      <c r="D49" s="7" t="inlineStr"/>
+          <t>Centrelink (Services Australia)</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Centrelink is a Services Australia program, not a separate legal entity.</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear fit — welfare/payments agency, not agriculture-sector focused.</t>
+        </is>
+      </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Lynk</t>
+          <t>https://www.servicesaustralia.gov.au/contact-us</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr"/>
-      <c r="G49" s="7" t="inlineStr"/>
-      <c r="H49" s="7" t="inlineStr"/>
-      <c r="I49" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>13 1272</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>Verified — fit weak</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Industry Body</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr"/>
-      <c r="D50" s="7" t="inlineStr"/>
+          <t>Department of Agriculture, Fisheries and Forestry (DAFF, Cwlth)</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Current name as of Jul 2022 (portfolio renamed repeatedly over the past decade — re-check periodically).</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Federal ag policy department — plausible commissioner/funder of large-scale producer survey work.</t>
+        </is>
+      </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>MLA (Meat &amp; Livestock Australia)</t>
+          <t>https://www.agriculture.gov.au</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr"/>
       <c r="G50" s="7" t="inlineStr"/>
-      <c r="H50" s="7" t="inlineStr"/>
-      <c r="I50" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Research/Market Research</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr"/>
-      <c r="D51" s="7" t="inlineStr"/>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>Morpace</t>
-        </is>
-      </c>
+          <t>National Water Commission</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Abolished by the National Water Commission (Abolition) Act 2015; functions moved to Productivity Commission.</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>N/A — defunct federal body, no current organisation to target.</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr"/>
       <c r="F51" s="7" t="inlineStr"/>
       <c r="G51" s="7" t="inlineStr"/>
-      <c r="H51" s="7" t="inlineStr"/>
-      <c r="I51" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>Not found — defunct</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Govt</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr"/>
-      <c r="D52" s="7" t="inlineStr"/>
+          <t>NSW Department of Primary Industries</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Folded into Department of Primary Industries and Regional Development (DPIRD NSW), 1 Jul 2024 — same entity researched in Target Accounts 2026.</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>State ag department — plausible buyer of grower/biosecurity survey data.</t>
+        </is>
+      </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>National Water Commission</t>
-        </is>
-      </c>
-      <c r="F52" s="7" t="inlineStr"/>
+          <t>https://www.dpird.nsw.gov.au/contact-us</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>contact@dpird.nsw.gov.au</t>
+        </is>
+      </c>
       <c r="G52" s="7" t="inlineStr"/>
-      <c r="H52" s="7" t="inlineStr"/>
-      <c r="I52" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Animal Health</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr"/>
-      <c r="D53" s="7" t="inlineStr"/>
+          <t>NSCA (National Safety Council of Australia)</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Now operates as NSCA Foundation, a WHS training/membership body.</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear fit for ag-specific data, though farm safety/WHS surveys plausible.</t>
+        </is>
+      </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Novartis (Animal Health)</t>
-        </is>
-      </c>
-      <c r="F53" s="7" t="inlineStr"/>
-      <c r="G53" s="7" t="inlineStr"/>
-      <c r="H53" s="7" t="inlineStr"/>
-      <c r="I53" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://nscafoundation.org.au/contact-the-nsca-foundation/</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>membership@nscafoundation.org.au</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>02 8875 7820</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>Ag Chem</t>
-        </is>
-      </c>
-      <c r="C54" s="7" t="inlineStr"/>
-      <c r="D54" s="7" t="inlineStr"/>
-      <c r="E54" s="7" t="inlineStr">
-        <is>
-          <t>Novozymes</t>
-        </is>
-      </c>
-      <c r="F54" s="7" t="inlineStr"/>
-      <c r="G54" s="7" t="inlineStr"/>
-      <c r="H54" s="7" t="inlineStr"/>
-      <c r="I54" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>University / research</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n"/>
+      <c r="C54" s="5" t="n"/>
+      <c r="D54" s="5" t="n"/>
+      <c r="E54" s="5" t="n"/>
+      <c r="F54" s="5" t="n"/>
+      <c r="G54" s="5" t="n"/>
+      <c r="H54" s="6" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C55" s="7" t="inlineStr"/>
-      <c r="D55" s="7" t="inlineStr"/>
+          <t>ACFR (Australian Centre for Field Robotics, Sydney Uni)</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Now sits under the broader Australian Centre for Robotics.</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear as a buyer — research centre, more likely a tech/data partner than a purchaser.</t>
+        </is>
+      </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>NSCA (National Safety Council of Australia)</t>
+          <t>http://www.acfr.usyd.edu.au/about/contact.shtml</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr"/>
-      <c r="G55" s="7" t="inlineStr"/>
-      <c r="H55" s="7" t="inlineStr"/>
-      <c r="I55" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>+61 2 9351 5549</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Industry Body</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="inlineStr"/>
-      <c r="D56" s="7" t="inlineStr"/>
+          <t>CQUniversity Australia</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear as a direct buyer — has ag-research programs but more likely a research partner.</t>
+        </is>
+      </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>NSW Farmers</t>
+          <t>https://www.cqu.edu.au/about-us/contacts</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr"/>
-      <c r="G56" s="7" t="inlineStr"/>
-      <c r="H56" s="7" t="inlineStr"/>
-      <c r="I56" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>1300 666 620</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Govt</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr"/>
-      <c r="D57" s="7" t="inlineStr"/>
+          <t>CSIRO</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>National science agency with a large Agriculture and Food division — plausible commissioner of structured data-collection work.</t>
+        </is>
+      </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>NSW Department of Primary Industries</t>
+          <t>https://www.csiro.au/en/contact</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr"/>
-      <c r="G57" s="7" t="inlineStr"/>
-      <c r="H57" s="7" t="inlineStr"/>
-      <c r="I57" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>1300 363 400</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Ag Chem</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="inlineStr"/>
-      <c r="D58" s="7" t="inlineStr"/>
+          <t>The University of Melbourne</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Ag sits within School of Agriculture, Food and Ecosystem Sciences (SAFES).</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Universities partner on ag extension/producer research and industry engagement — plausible buyer/collaborator.</t>
+        </is>
+      </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>Nufarm</t>
-        </is>
-      </c>
-      <c r="F58" s="7" t="inlineStr"/>
-      <c r="G58" s="7" t="inlineStr"/>
-      <c r="H58" s="7" t="inlineStr"/>
-      <c r="I58" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://safes.unimelb.edu.au/about/contact-us</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>darren.coomber@unimelb.edu.au</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>+61 3 9035 5024</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="C59" s="7" t="inlineStr"/>
-      <c r="D59" s="7" t="inlineStr"/>
+          <t>The University of Sydney</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Ag research consolidated under Sydney Institute of Agriculture.</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Same rationale as Melbourne.</t>
+        </is>
+      </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>OneSteel</t>
-        </is>
-      </c>
-      <c r="F59" s="7" t="inlineStr"/>
-      <c r="G59" s="7" t="inlineStr"/>
-      <c r="H59" s="7" t="inlineStr"/>
-      <c r="I59" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://www.sydney.edu.au/agriculture/about/contact-and-locations.html</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>soles.hos@sydney.edu.au</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>+61 2 9351 2848</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Fin/Ins</t>
-        </is>
-      </c>
-      <c r="C60" s="7" t="inlineStr"/>
-      <c r="D60" s="7" t="inlineStr"/>
+          <t>University of Wollongong Australia</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear fit — not a notable agricultural research institution.</t>
+        </is>
+      </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>Oxley Capital Partners</t>
-        </is>
-      </c>
-      <c r="F60" s="7" t="inlineStr"/>
-      <c r="G60" s="7" t="inlineStr"/>
-      <c r="H60" s="7" t="inlineStr"/>
-      <c r="I60" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://www.uow.edu.au/about/contacts/</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>askuow@uow.edu.au</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>1300 275 869</t>
+        </is>
+      </c>
+      <c r="H60" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B61" s="7" t="inlineStr">
-        <is>
-          <t>Animal Health</t>
-        </is>
-      </c>
-      <c r="C61" s="7" t="inlineStr"/>
-      <c r="D61" s="7" t="inlineStr"/>
-      <c r="E61" s="7" t="inlineStr">
-        <is>
-          <t>Pfizer (Animal Health)</t>
-        </is>
-      </c>
-      <c r="F61" s="7" t="inlineStr"/>
-      <c r="G61" s="7" t="inlineStr"/>
-      <c r="H61" s="7" t="inlineStr"/>
-      <c r="I61" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>AgTech</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="n"/>
+      <c r="C61" s="5" t="n"/>
+      <c r="D61" s="5" t="n"/>
+      <c r="E61" s="5" t="n"/>
+      <c r="F61" s="5" t="n"/>
+      <c r="G61" s="5" t="n"/>
+      <c r="H61" s="6" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Machinery</t>
-        </is>
-      </c>
-      <c r="C62" s="7" t="inlineStr"/>
-      <c r="D62" s="7" t="inlineStr"/>
-      <c r="E62" s="7" t="inlineStr">
-        <is>
-          <t>Philmac</t>
-        </is>
-      </c>
+          <t>CropLogic</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>Defunct in ag — suspended 2019, reverse takeover, renamed Olympio Metals Ltd (ASX:OLY) in 2022, now a WA mineral exploration company.</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>N/A — no longer operates in agriculture.</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr"/>
       <c r="F62" s="7" t="inlineStr"/>
       <c r="G62" s="7" t="inlineStr"/>
-      <c r="H62" s="7" t="inlineStr"/>
-      <c r="I62" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>Not found — defunct</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Industry Body</t>
-        </is>
-      </c>
-      <c r="C63" s="7" t="inlineStr"/>
-      <c r="D63" s="7" t="inlineStr"/>
+          <t>FarmBot Monitoring Solutions</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — Sydney-based, ~8,000+ farmer customers, Telstra/Macdoch Ventures backed.</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Agtech IoT vendor already selling data services to farmers — plausible partner or customer for structured phone-data workflows.</t>
+        </is>
+      </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>Plant Health Australia</t>
-        </is>
-      </c>
-      <c r="F63" s="7" t="inlineStr"/>
-      <c r="G63" s="7" t="inlineStr"/>
-      <c r="H63" s="7" t="inlineStr"/>
-      <c r="I63" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://farmbot.com.au/contact-us/</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>info@farmbot.com.au</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>02 9030 4760</t>
+        </is>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Research/Market Research</t>
-        </is>
-      </c>
-      <c r="C64" s="7" t="inlineStr"/>
-      <c r="D64" s="7" t="inlineStr"/>
+          <t>IPSTAR Broadband</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>Still active, now largely an NBN Sky Muster reseller for rural connectivity.</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Weak/moderate fit — shares the same rural-Australia customer base, could care about connectivity/usage research.</t>
+        </is>
+      </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>Power Stats</t>
+          <t>https://ipstarbroadband.com.au/get-in-touch/</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr"/>
-      <c r="G64" s="7" t="inlineStr"/>
-      <c r="H64" s="7" t="inlineStr"/>
-      <c r="I64" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>1800 477 827</t>
+        </is>
+      </c>
+      <c r="H64" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>AgTech</t>
-        </is>
-      </c>
-      <c r="C65" s="7" t="inlineStr"/>
-      <c r="D65" s="7" t="inlineStr"/>
+          <t>Precision Ag Solutions</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged — Toowoomba, QLD precision-ag dealer.</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear — sells hardware/support, not a natural data-services buyer, though dealer/customer satisfaction surveys conceivable.</t>
+        </is>
+      </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Precision Ag Solutions</t>
-        </is>
-      </c>
-      <c r="F65" s="7" t="inlineStr"/>
-      <c r="G65" s="7" t="inlineStr"/>
-      <c r="H65" s="7" t="inlineStr"/>
-      <c r="I65" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://www.precisionagsolutions.com.au/contact</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>info@precisionagsolutions.com.au</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>1800 497 032</t>
+        </is>
+      </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B66" s="7" t="inlineStr">
-        <is>
-          <t>Govt</t>
-        </is>
-      </c>
-      <c r="C66" s="7" t="inlineStr"/>
-      <c r="D66" s="7" t="inlineStr"/>
-      <c r="E66" s="7" t="inlineStr">
-        <is>
-          <t>Queensland Government - Dept of Agriculture and Fisheries</t>
-        </is>
-      </c>
-      <c r="F66" s="7" t="inlineStr"/>
-      <c r="G66" s="7" t="inlineStr"/>
-      <c r="H66" s="7" t="inlineStr"/>
-      <c r="I66" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>Media, research &amp; tech peers (potential partners, not necessarily buyers)</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="n"/>
+      <c r="C66" s="5" t="n"/>
+      <c r="D66" s="5" t="n"/>
+      <c r="E66" s="5" t="n"/>
+      <c r="F66" s="5" t="n"/>
+      <c r="G66" s="5" t="n"/>
+      <c r="H66" s="6" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Research/Market Research</t>
-        </is>
-      </c>
-      <c r="C67" s="7" t="inlineStr"/>
-      <c r="D67" s="7" t="inlineStr"/>
+          <t>AUSTAR</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>Defunct as standalone brand — merged into Foxtel by 2014.</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear — was a pay-TV operator; no clear agri-data rationale.</t>
+        </is>
+      </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Red Handed (Communications Group)</t>
+          <t>https://www.foxtel.com.au</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr"/>
       <c r="G67" s="7" t="inlineStr"/>
-      <c r="H67" s="7" t="inlineStr"/>
-      <c r="I67" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>Not found — defunct, successor Foxtel</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Research/Market Research</t>
-        </is>
-      </c>
-      <c r="C68" s="7" t="inlineStr"/>
-      <c r="D68" s="7" t="inlineStr"/>
-      <c r="E68" s="7" t="inlineStr">
-        <is>
-          <t>RGA</t>
-        </is>
-      </c>
+          <t>Food Industry People Group</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>Acquired by ASX-listed PeopleIN ($45M); QLD-based food-industry/FMCG labour-hire and workforce recruiter.</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear — labour supply, not obviously an ag-data buyer.</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr"/>
       <c r="F68" s="7" t="inlineStr"/>
       <c r="G68" s="7" t="inlineStr"/>
-      <c r="H68" s="7" t="inlineStr"/>
-      <c r="I68" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H68" s="7" t="inlineStr">
+        <is>
+          <t>Not found</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C69" s="7" t="inlineStr"/>
-      <c r="D69" s="7" t="inlineStr"/>
+          <t>Kantar</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — global market-research group, owned by Bain Capital since 2019.</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Plausible as a peer/partnership target — a market-research firm that could resell or white-label phone-survey data collection, not an end customer.</t>
+        </is>
+      </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>Riverbank Redlands</t>
+          <t>https://kantaraustralia.com/contact/</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr"/>
       <c r="G69" s="7" t="inlineStr"/>
-      <c r="H69" s="7" t="inlineStr"/>
-      <c r="I69" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="inlineStr"/>
-      <c r="D70" s="7" t="inlineStr"/>
+          <t>Morpace</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Merged with Market Strategies International, relaunched as Escalent (May 2019); Morpace brand largely discontinued.</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>N/A as standalone entity — successor Escalent is a US-based human-behavior/analytics research firm, not ag-specific.</t>
+        </is>
+      </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>Ruralco Insurance</t>
+          <t>https://escalent.co</t>
         </is>
       </c>
       <c r="F70" s="7" t="inlineStr"/>
       <c r="G70" s="7" t="inlineStr"/>
-      <c r="H70" s="7" t="inlineStr"/>
-      <c r="I70" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Industry Body</t>
-        </is>
-      </c>
-      <c r="C71" s="7" t="inlineStr"/>
-      <c r="D71" s="7" t="inlineStr"/>
+          <t>Power Stats</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged — Sydney statistical consulting firm since 2002.</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear as end-buyer — analytics subcontractor to market-research/ad agencies, more plausible as partner/competitor.</t>
+        </is>
+      </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>Sheep Producers Australia</t>
-        </is>
-      </c>
-      <c r="F71" s="7" t="inlineStr"/>
-      <c r="G71" s="7" t="inlineStr"/>
-      <c r="H71" s="7" t="inlineStr"/>
-      <c r="I71" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://powerstats.com.au/contact/</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>enquiries@powerstats.com.au</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>+61 2 9804 0271</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Machinery</t>
-        </is>
-      </c>
-      <c r="C72" s="7" t="inlineStr"/>
-      <c r="D72" s="7" t="inlineStr"/>
+          <t>Red Handed (Communications Group)</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Rebranded — now trades as Redhanded (Redhanded Creative), Clemenger Group holds a strategic stake.</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>B2B/rural media and research agency for regional/agricultural audiences — more likely a channel partner or referral source than an end buyer.</t>
+        </is>
+      </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>Silvan</t>
-        </is>
-      </c>
-      <c r="F72" s="7" t="inlineStr"/>
-      <c r="G72" s="7" t="inlineStr"/>
-      <c r="H72" s="7" t="inlineStr"/>
-      <c r="I72" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://redhanded.com.au/</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>social@redhanded.com.au</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>+61 3 9917 3430</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Ag Chem</t>
-        </is>
-      </c>
-      <c r="C73" s="7" t="inlineStr"/>
-      <c r="D73" s="7" t="inlineStr"/>
+          <t>Taverner Research</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — full-service Australian market research firm.</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Itself a market-research/data-collection firm — more relevant as a potential competitor/subcontract partner than an end customer.</t>
+        </is>
+      </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Sinochem Australia</t>
-        </is>
-      </c>
-      <c r="F73" s="7" t="inlineStr"/>
-      <c r="G73" s="7" t="inlineStr"/>
-      <c r="H73" s="7" t="inlineStr"/>
-      <c r="I73" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://taverner.com.au/contact-us/</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>research@taverner.com.au</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>(02) 9212 2900</t>
+        </is>
+      </c>
+      <c r="H73" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="C74" s="7" t="inlineStr"/>
-      <c r="D74" s="7" t="inlineStr"/>
+          <t>hlt (Healthy Thinking)</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>Now Healthy Thinking Group, healthcare advertising/comms agency.</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear fit — health-sector focused, not agriculture.</t>
+        </is>
+      </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>Smorgon Steel</t>
+          <t>https://www.healthythinkinggroup.com/contact</t>
         </is>
       </c>
       <c r="F74" s="7" t="inlineStr"/>
-      <c r="G74" s="7" t="inlineStr"/>
-      <c r="H74" s="7" t="inlineStr"/>
-      <c r="I74" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>+61 404 876 000</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Ag Chem</t>
-        </is>
-      </c>
-      <c r="C75" s="7" t="inlineStr"/>
-      <c r="D75" s="7" t="inlineStr"/>
+          <t>The Weekly Times</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — News Corp Australia's rural newspaper, national rural readership.</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Rural media outlet — natural interest in reader/producer research and content partnerships.</t>
+        </is>
+      </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>Sumitomo Chemical</t>
-        </is>
-      </c>
-      <c r="F75" s="7" t="inlineStr"/>
-      <c r="G75" s="7" t="inlineStr"/>
-      <c r="H75" s="7" t="inlineStr"/>
-      <c r="I75" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://www.weeklytimes.com.au/</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>online@theweeklytimes.com.au</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>+61 3 9292 2000</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>Machinery</t>
-        </is>
-      </c>
-      <c r="C76" s="7" t="inlineStr"/>
-      <c r="D76" s="7" t="inlineStr"/>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged.</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear — touched agri-AI before (Watson Decision Platform for Agriculture, discontinued ~2021); more plausible as a tech partner/competitor than customer.</t>
+        </is>
+      </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>Tapex</t>
+          <t>https://www.ibm.com/au-en/contact</t>
         </is>
       </c>
       <c r="F76" s="7" t="inlineStr"/>
-      <c r="G76" s="7" t="inlineStr"/>
-      <c r="H76" s="7" t="inlineStr"/>
-      <c r="I76" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>13 2426</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>Research/Market Research</t>
-        </is>
-      </c>
-      <c r="C77" s="7" t="inlineStr"/>
-      <c r="D77" s="7" t="inlineStr"/>
+          <t>Lynk</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Identity unverified — best match found is Lynk Global (Hong Kong/Singapore expert-network platform); could not confirm this is the same "Lynk" from the logo. Re-check the original logo before outreach.</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>If correct, plausible as a competitor/subcontracting partner for structured data collection, not agriculture-specific.</t>
+        </is>
+      </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>Taverner Research</t>
+          <t>https://lynk.global</t>
         </is>
       </c>
       <c r="F77" s="7" t="inlineStr"/>
       <c r="G77" s="7" t="inlineStr"/>
-      <c r="H77" s="7" t="inlineStr"/>
-      <c r="I77" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>Not found — identity unverified</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B78" s="7" t="inlineStr">
-        <is>
-          <t>Research/Market Research</t>
-        </is>
-      </c>
-      <c r="C78" s="7" t="inlineStr"/>
-      <c r="D78" s="7" t="inlineStr"/>
-      <c r="E78" s="7" t="inlineStr">
-        <is>
-          <t>hlt (Healthy Thinking)</t>
-        </is>
-      </c>
-      <c r="F78" s="7" t="inlineStr"/>
-      <c r="G78" s="7" t="inlineStr"/>
-      <c r="H78" s="7" t="inlineStr"/>
-      <c r="I78" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>Banks</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="n"/>
+      <c r="C78" s="5" t="n"/>
+      <c r="D78" s="5" t="n"/>
+      <c r="E78" s="5" t="n"/>
+      <c r="F78" s="5" t="n"/>
+      <c r="G78" s="5" t="n"/>
+      <c r="H78" s="6" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>University/Research</t>
-        </is>
-      </c>
-      <c r="C79" s="7" t="inlineStr"/>
-      <c r="D79" s="7" t="inlineStr"/>
+          <t>ANZ</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged. Also covered in Target Accounts 2026 — reconcile before outreach to avoid duplicate contact.</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Agribusiness banking arm could use structured farmer-outreach/data collection for credit/relationship insights.</t>
+        </is>
+      </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>The University of Melbourne</t>
+          <t>https://www.anz.com.au/business/industries/agribusiness/</t>
         </is>
       </c>
       <c r="F79" s="7" t="inlineStr"/>
       <c r="G79" s="7" t="inlineStr"/>
-      <c r="H79" s="7" t="inlineStr"/>
-      <c r="I79" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B80" s="7" t="inlineStr">
-        <is>
-          <t>University/Research</t>
-        </is>
-      </c>
-      <c r="C80" s="7" t="inlineStr"/>
-      <c r="D80" s="7" t="inlineStr"/>
-      <c r="E80" s="7" t="inlineStr">
-        <is>
-          <t>The University of Sydney</t>
-        </is>
-      </c>
-      <c r="F80" s="7" t="inlineStr"/>
-      <c r="G80" s="7" t="inlineStr"/>
-      <c r="H80" s="7" t="inlineStr"/>
-      <c r="I80" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>Grain (legacy / defunct)</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="n"/>
+      <c r="C80" s="5" t="n"/>
+      <c r="D80" s="5" t="n"/>
+      <c r="E80" s="5" t="n"/>
+      <c r="F80" s="5" t="n"/>
+      <c r="G80" s="5" t="n"/>
+      <c r="H80" s="6" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>University/Research</t>
-        </is>
-      </c>
-      <c r="C81" s="7" t="inlineStr"/>
-      <c r="D81" s="7" t="inlineStr"/>
-      <c r="E81" s="7" t="inlineStr">
-        <is>
-          <t>University of Wollongong Australia</t>
-        </is>
-      </c>
+          <t>AWB</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>Defunct as standalone company. Rural services arm (Landmark) sold to Agrium in 2010 (now Nutrien Ag Solutions); grain trading/storage arm became AWB Grainflow, subsidiary of Cargill Australia.</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>N/A — folded into successor entities (see Nutrien Ag Solutions / Cargill in Target Accounts 2026).</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr"/>
       <c r="F81" s="7" t="inlineStr"/>
       <c r="G81" s="7" t="inlineStr"/>
-      <c r="H81" s="7" t="inlineStr"/>
-      <c r="I81" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>Not found — defunct</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B82" s="7" t="inlineStr">
-        <is>
-          <t>Machinery</t>
-        </is>
-      </c>
-      <c r="C82" s="7" t="inlineStr"/>
-      <c r="D82" s="7" t="inlineStr"/>
-      <c r="E82" s="7" t="inlineStr">
-        <is>
-          <t>Toyota</t>
-        </is>
-      </c>
-      <c r="F82" s="7" t="inlineStr"/>
-      <c r="G82" s="7" t="inlineStr"/>
-      <c r="H82" s="7" t="inlineStr"/>
-      <c r="I82" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>Industrial / other</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="n"/>
+      <c r="C82" s="5" t="n"/>
+      <c r="D82" s="5" t="n"/>
+      <c r="E82" s="5" t="n"/>
+      <c r="F82" s="5" t="n"/>
+      <c r="G82" s="5" t="n"/>
+      <c r="H82" s="6" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C83" s="7" t="inlineStr"/>
-      <c r="D83" s="7" t="inlineStr"/>
+          <t>BHP Group (formerly BHP Billiton)</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Renamed BHP Group, effective 19 Nov 2018.</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear — mining major, no direct agriculture connection (historical potash/fertiliser interest via Jansen, not core).</t>
+        </is>
+      </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>The Weekly Times</t>
+          <t>https://www.bhp.com/contact-us</t>
         </is>
       </c>
       <c r="F83" s="7" t="inlineStr"/>
       <c r="G83" s="7" t="inlineStr"/>
-      <c r="H83" s="7" t="inlineStr"/>
-      <c r="I83" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>Verified — fit weak</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C84" s="7" t="inlineStr"/>
-      <c r="D84" s="7" t="inlineStr"/>
+          <t>Ampol (formerly Caltex Australia)</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>Renamed Ampol Limited, May 2020, full brand transition by end of 2022.</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear — fuel retailer/distributor; rural fuel card business is the closest tie to agriculture.</t>
+        </is>
+      </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>Valiant</t>
+          <t>https://www.ampol.com.au/about-ampol/news-and-media/contact</t>
         </is>
       </c>
       <c r="F84" s="7" t="inlineStr"/>
       <c r="G84" s="7" t="inlineStr"/>
-      <c r="H84" s="7" t="inlineStr"/>
-      <c r="I84" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H84" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>Industry Body</t>
-        </is>
-      </c>
-      <c r="C85" s="7" t="inlineStr"/>
-      <c r="D85" s="7" t="inlineStr"/>
+          <t>OneSteel</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Renamed Arrium (2012); Arrium collapsed 2016, long-products business bought by GFG Alliance/Liberty, now InfraBuild.</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear — steel manufacturer/distributor, only tangential ag relevance (rural fencing/wire).</t>
+        </is>
+      </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>Victorian Farmers Federation</t>
-        </is>
-      </c>
-      <c r="F85" s="7" t="inlineStr"/>
-      <c r="G85" s="7" t="inlineStr"/>
-      <c r="H85" s="7" t="inlineStr"/>
-      <c r="I85" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+          <t>https://www.infrabuild.com/contact-us/</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>sustainablesteel@infrabuild.com</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="inlineStr">
+        <is>
+          <t>02 8424 9800</t>
+        </is>
+      </c>
+      <c r="H85" s="7" t="inlineStr">
+        <is>
+          <t>Verified — successor entity</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>Animal Health</t>
-        </is>
-      </c>
-      <c r="C86" s="7" t="inlineStr"/>
-      <c r="D86" s="7" t="inlineStr"/>
+          <t>Smorgon Steel</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>Defunct as independent company — acquired by Arrium/OneSteel (2007); Arrium collapsed 2016, now InfraBuild (same successor as OneSteel above).</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear — industrial steel/scrap recycler, only tangential ag relevance.</t>
+        </is>
+      </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>Virbac</t>
+          <t>https://www.infrabuild.com/contact-us/</t>
         </is>
       </c>
       <c r="F86" s="7" t="inlineStr"/>
       <c r="G86" s="7" t="inlineStr"/>
-      <c r="H86" s="7" t="inlineStr"/>
-      <c r="I86" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="H86" s="7" t="inlineStr">
+        <is>
+          <t>Partial — original entity defunct</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>Agribus</t>
-        </is>
-      </c>
-      <c r="C87" s="7" t="inlineStr"/>
-      <c r="D87" s="7" t="inlineStr"/>
+          <t>CopRice</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — animal feed brand of Ridley Corporation.</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>Livestock feed manufacturer — could use farmer feedback/ordering data.</t>
+        </is>
+      </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
+          <t>https://www.coprice.com.au/contact/</t>
+        </is>
+      </c>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>sales@coprice.com.au</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>1800 029 901</t>
+        </is>
+      </c>
+      <c r="H87" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>Oxley Capital Partners</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>Unchanged — Sydney food/agribusiness corporate advisory and investment firm.</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="inlineStr">
+        <is>
+          <t>Agribusiness M&amp;A advisory shop — could value structured on-farm/market data for deal due diligence and sector intelligence.</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>https://oxleycp.com/contact/</t>
+        </is>
+      </c>
+      <c r="F88" s="7" t="inlineStr">
+        <is>
+          <t>info@oxleycp.com</t>
+        </is>
+      </c>
+      <c r="G88" s="7" t="inlineStr">
+        <is>
+          <t>(02) 9083 2173</t>
+        </is>
+      </c>
+      <c r="H88" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="7" t="inlineStr">
+        <is>
           <t>Wesfarmers</t>
         </is>
       </c>
-      <c r="F87" s="7" t="inlineStr"/>
-      <c r="G87" s="7" t="inlineStr"/>
-      <c r="H87" s="7" t="inlineStr"/>
-      <c r="I87" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B88" s="7" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="C88" s="7" t="inlineStr"/>
-      <c r="D88" s="7" t="inlineStr"/>
-      <c r="E88" s="7" t="inlineStr">
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged — diversified conglomerate.</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear at parent level — no longer has a direct ag-services division (sold Landmark years ago); only tangential relevance via CSBP.</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr">
+        <is>
+          <t>https://www.wesfarmers.com.au/util/contact</t>
+        </is>
+      </c>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>debt@wesfarmers.com.au (debt investors only)</t>
+        </is>
+      </c>
+      <c r="G89" s="7" t="inlineStr"/>
+      <c r="H89" s="7" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>Greening Australia</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged — still operating independently, national environmental restoration NGO.</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Weak/unclear for ag phone-survey product, though plausible for landholder/revegetation-program data collection.</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>https://www.greeningaustralia.org.au/contact/</t>
+        </is>
+      </c>
+      <c r="F90" s="7" t="inlineStr">
+        <is>
+          <t>info@greeningaustralia.org.au</t>
+        </is>
+      </c>
+      <c r="G90" s="7" t="inlineStr">
+        <is>
+          <t>1300 886 589</t>
+        </is>
+      </c>
+      <c r="H90" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>Heritage Seeds</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>Appears to still trade independently (heritageseeds.com.au); ownership status uncertain — could not confirm acquisition claims.</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>Seed company — could buy grower feedback/trial data.</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>https://heritageseeds.com.au</t>
+        </is>
+      </c>
+      <c r="F91" s="7" t="inlineStr"/>
+      <c r="G91" s="7" t="inlineStr">
+        <is>
+          <t>03 9501 7000</t>
+        </is>
+      </c>
+      <c r="H91" s="7" t="inlineStr">
+        <is>
+          <t>Partial — ownership uncertain</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>Riverbank Redlands</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>Could not identify a current or historical organisation matching this exact name (searched nursery, turf, oyster, poultry, real-estate angles).</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>Unable to confirm fit — identity unresolved.</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr"/>
+      <c r="F92" s="7" t="inlineStr"/>
+      <c r="G92" s="7" t="inlineStr"/>
+      <c r="H92" s="7" t="inlineStr">
+        <is>
+          <t>Not found — unidentified, re-check original logo</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Valiant</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>Ambiguous — candidates include Valiant Power (solar light towers), Valiant Finance (SME/ag equipment lending), Valiant Hire (furniture), or the defunct Chrysler Valiant brand.</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>Fit unclear given name ambiguity — cannot assign rationale without confirming the entity.</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr"/>
+      <c r="F93" s="7" t="inlineStr"/>
+      <c r="G93" s="7" t="inlineStr"/>
+      <c r="H93" s="7" t="inlineStr">
+        <is>
+          <t>Not found — identity unresolved, re-check original logo</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>Already covered in Target Accounts 2026 (not re-researched)</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="n"/>
+      <c r="C94" s="5" t="n"/>
+      <c r="D94" s="5" t="n"/>
+      <c r="E94" s="5" t="n"/>
+      <c r="F94" s="5" t="n"/>
+      <c r="G94" s="5" t="n"/>
+      <c r="H94" s="6" t="n"/>
+    </row>
+    <row r="95">
+      <c r="B95" s="12" t="inlineStr">
+        <is>
+          <t>Cargill</t>
+        </is>
+      </c>
+      <c r="C95" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate — see Target Accounts 2026, "Grain buyers / handlers / traders".</t>
+        </is>
+      </c>
+      <c r="D95" s="12" t="inlineStr"/>
+      <c r="E95" s="12" t="inlineStr"/>
+      <c r="F95" s="12" t="inlineStr"/>
+      <c r="G95" s="12" t="inlineStr"/>
+      <c r="H95" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" s="12" t="inlineStr">
+        <is>
+          <t>Clear Grain Exchange</t>
+        </is>
+      </c>
+      <c r="C96" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate — see Target Accounts 2026.</t>
+        </is>
+      </c>
+      <c r="D96" s="12" t="inlineStr"/>
+      <c r="E96" s="12" t="inlineStr"/>
+      <c r="F96" s="12" t="inlineStr"/>
+      <c r="G96" s="12" t="inlineStr"/>
+      <c r="H96" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="12" t="inlineStr">
+        <is>
+          <t>Commonwealth Bank</t>
+        </is>
+      </c>
+      <c r="C97" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate — see Target Accounts 2026, "Banks".</t>
+        </is>
+      </c>
+      <c r="D97" s="12" t="inlineStr"/>
+      <c r="E97" s="12" t="inlineStr"/>
+      <c r="F97" s="12" t="inlineStr"/>
+      <c r="G97" s="12" t="inlineStr"/>
+      <c r="H97" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" s="12" t="inlineStr">
+        <is>
+          <t>Elders</t>
+        </is>
+      </c>
+      <c r="C98" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate — see Target Accounts 2026, "Ag retail / input suppliers".</t>
+        </is>
+      </c>
+      <c r="D98" s="12" t="inlineStr"/>
+      <c r="E98" s="12" t="inlineStr"/>
+      <c r="F98" s="12" t="inlineStr"/>
+      <c r="G98" s="12" t="inlineStr"/>
+      <c r="H98" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="12" t="inlineStr">
+        <is>
+          <t>GrainCorp</t>
+        </is>
+      </c>
+      <c r="C99" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate — see Target Accounts 2026.</t>
+        </is>
+      </c>
+      <c r="D99" s="12" t="inlineStr"/>
+      <c r="E99" s="12" t="inlineStr"/>
+      <c r="F99" s="12" t="inlineStr"/>
+      <c r="G99" s="12" t="inlineStr"/>
+      <c r="H99" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" s="12" t="inlineStr">
+        <is>
+          <t>GRDC</t>
+        </is>
+      </c>
+      <c r="C100" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate — see Target Accounts 2026, "Government / research / industry bodies".</t>
+        </is>
+      </c>
+      <c r="D100" s="12" t="inlineStr"/>
+      <c r="E100" s="12" t="inlineStr"/>
+      <c r="F100" s="12" t="inlineStr"/>
+      <c r="G100" s="12" t="inlineStr"/>
+      <c r="H100" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="12" t="inlineStr">
+        <is>
+          <t>Landmark</t>
+        </is>
+      </c>
+      <c r="C101" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate — now Nutrien Ag Solutions, see Target Accounts 2026.</t>
+        </is>
+      </c>
+      <c r="D101" s="12" t="inlineStr"/>
+      <c r="E101" s="12" t="inlineStr"/>
+      <c r="F101" s="12" t="inlineStr"/>
+      <c r="G101" s="12" t="inlineStr"/>
+      <c r="H101" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" s="12" t="inlineStr">
+        <is>
+          <t>Queensland Government — Dept of Agriculture and Fisheries</t>
+        </is>
+      </c>
+      <c r="C102" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate — now QLD Dept of Primary Industries (DPI), see Target Accounts 2026.</t>
+        </is>
+      </c>
+      <c r="D102" s="12" t="inlineStr"/>
+      <c r="E102" s="12" t="inlineStr"/>
+      <c r="F102" s="12" t="inlineStr"/>
+      <c r="G102" s="12" t="inlineStr"/>
+      <c r="H102" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" s="12" t="inlineStr">
         <is>
           <t>WFI Insurance</t>
         </is>
       </c>
-      <c r="F88" s="7" t="inlineStr"/>
-      <c r="G88" s="7" t="inlineStr"/>
-      <c r="H88" s="7" t="inlineStr"/>
-      <c r="I88" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B89" s="7" t="inlineStr">
-        <is>
-          <t>Insurance</t>
-        </is>
-      </c>
-      <c r="C89" s="7" t="inlineStr"/>
-      <c r="D89" s="7" t="inlineStr"/>
-      <c r="E89" s="7" t="inlineStr">
-        <is>
-          <t>WorkCover SA</t>
-        </is>
-      </c>
-      <c r="F89" s="7" t="inlineStr"/>
-      <c r="G89" s="7" t="inlineStr"/>
-      <c r="H89" s="7" t="inlineStr"/>
-      <c r="I89" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="7" t="inlineStr">
-        <is>
-          <t>Client wall</t>
-        </is>
-      </c>
-      <c r="B90" s="7" t="inlineStr">
-        <is>
-          <t>Animal Health</t>
-        </is>
-      </c>
-      <c r="C90" s="7" t="inlineStr"/>
-      <c r="D90" s="7" t="inlineStr"/>
-      <c r="E90" s="7" t="inlineStr">
-        <is>
-          <t>Zoetis</t>
-        </is>
-      </c>
-      <c r="F90" s="7" t="inlineStr"/>
-      <c r="G90" s="7" t="inlineStr"/>
-      <c r="H90" s="7" t="inlineStr"/>
-      <c r="I90" s="7" t="inlineStr">
-        <is>
-          <t>From uploaded client-wall image; contact details not yet researched.</t>
+      <c r="C103" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate — see Target Accounts 2026, "Insurers".</t>
+        </is>
+      </c>
+      <c r="D103" s="12" t="inlineStr"/>
+      <c r="E103" s="12" t="inlineStr"/>
+      <c r="F103" s="12" t="inlineStr"/>
+      <c r="G103" s="12" t="inlineStr"/>
+      <c r="H103" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+  <mergeCells count="15">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A80:H80"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A78:H78"/>
+    <mergeCell ref="A94:H94"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A54:H54"/>
+    <mergeCell ref="A82:H82"/>
+    <mergeCell ref="A66:H66"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A61:H61"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>